<commit_message>
nouveau template METROLOGO freq
</commit_message>
<xml_diff>
--- a/Templates/METROLOGO.xlsx
+++ b/Templates/METROLOGO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GLB\Desktop\projet\MetrologoWPF\MetrologoWPF\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{132DF534-6383-4265-B30D-06A81A0A789B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC58DC2B-846A-4047-BE5F-82DB8A03CAF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="2610" windowWidth="26685" windowHeight="14085" xr2:uid="{05031086-6F6F-4E7A-BF9B-F73FC503154F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{05031086-6F6F-4E7A-BF9B-F73FC503154F}"/>
   </bookViews>
   <sheets>
     <sheet name="ModFeuille" sheetId="1" r:id="rId1"/>
@@ -984,7 +984,7 @@
         <v>7</v>
       </c>
       <c r="C29" s="6">
-        <f>IF(ISBLANK(ZNCoeffB),,(IF(ISBLANK(ZNFreqMoyReel),,ZNCoeffB/ZNFreqMoyReel+ZNCoeffA)))</f>
+        <f>IF(ISBLANK(ZNCoeffB),,(IF(ISBLANK(ZNFreqMoyReel),,SQRT((ZNCoeffB/ZNFreqMoyReel)^2+(ZNCoeffA)^2))))</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>